<commit_message>
Changed supported endpoints for end user Graph
</commit_message>
<xml_diff>
--- a/Supported Endpoints/Full API List.xlsx
+++ b/Supported Endpoints/Full API List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tdworldwide.sharepoint.com/sites/CloudSalesEngineering/Shared Documents/Microsoft Azure/PAC Proxy/Bulk Upload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="714" documentId="11_1EF87C37D373E2B26C3EB6EE3A64704C51DC5438" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8FB597A-DC00-4964-8347-6C8D41ABC178}"/>
+  <xr:revisionPtr revIDLastSave="730" documentId="11_1EF87C37D373E2B26C3EB6EE3A64704C51DC5438" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA977F14-2CB1-417B-B5DE-91F875E48197}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2323" uniqueCount="890">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2316" uniqueCount="890">
   <si>
     <t>Oid</t>
   </si>
@@ -3277,12 +3277,10 @@
         <v>16</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="1" t="s">
-        <v>531</v>
-      </c>
+      <c r="E4" s="1"/>
       <c r="F4" s="1" t="s">
         <v>17</v>
       </c>
@@ -6166,12 +6164,10 @@
         <v>287</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D97" s="1"/>
-      <c r="E97" s="1" t="s">
-        <v>531</v>
-      </c>
+      <c r="E97" s="1"/>
       <c r="F97" s="1" t="s">
         <v>17</v>
       </c>
@@ -6228,12 +6224,10 @@
         <v>293</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D99" s="1"/>
-      <c r="E99" s="1" t="s">
-        <v>531</v>
-      </c>
+      <c r="E99" s="1"/>
       <c r="F99" s="1" t="s">
         <v>17</v>
       </c>
@@ -6259,12 +6253,10 @@
         <v>296</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D100" s="1"/>
-      <c r="E100" s="1" t="s">
-        <v>531</v>
-      </c>
+      <c r="E100" s="1"/>
       <c r="F100" s="1" t="s">
         <v>17</v>
       </c>
@@ -6290,12 +6282,10 @@
         <v>299</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D101" s="1"/>
-      <c r="E101" s="1" t="s">
-        <v>531</v>
-      </c>
+      <c r="E101" s="1"/>
       <c r="F101" s="1" t="s">
         <v>17</v>
       </c>
@@ -6321,12 +6311,10 @@
         <v>302</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D102" s="1"/>
-      <c r="E102" s="1" t="s">
-        <v>531</v>
-      </c>
+      <c r="E102" s="1"/>
       <c r="F102" s="1" t="s">
         <v>17</v>
       </c>
@@ -6352,12 +6340,10 @@
         <v>305</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D103" s="1"/>
-      <c r="E103" s="1" t="s">
-        <v>531</v>
-      </c>
+      <c r="E103" s="1"/>
       <c r="F103" s="1" t="s">
         <v>17</v>
       </c>

</xml_diff>